<commit_message>
Release btp_si_compare_2026.xlsx: video YouTube live
</commit_message>
<xml_diff>
--- a/simulatori/btp_si_compare_2026.xlsx
+++ b/simulatori/btp_si_compare_2026.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="0 - Indice" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1 - Parametri" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2 - BTP Italia Si" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3 - BTP Italia classico" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="4 - BTP Valore" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="5 - BTP Futura" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="6 - BTP nominali" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="7 - MATRICE COMPARATIVA" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="8 - Break-even" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="9 - 4 profili FIRE" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10 - Calcolatore personale" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0 - Indice" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 - Parametri" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 - BTP Italia Si" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 - BTP Italia classico" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 - BTP Valore" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 - BTP Futura" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 - BTP nominali" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 - MATRICE COMPARATIVA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 - Break-even" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 - 4 profili FIRE" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 - Calcolatore personale" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -279,14 +279,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -311,7 +311,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -352,7 +352,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -363,8 +363,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -404,14 +404,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -436,7 +436,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -477,7 +477,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -488,8 +488,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -529,14 +529,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -561,7 +561,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -602,7 +602,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -613,8 +613,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -654,14 +654,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -686,7 +686,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -727,7 +727,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -738,8 +738,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -779,14 +779,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -810,14 +810,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -846,8 +846,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -884,7 +884,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -895,8 +895,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -936,14 +936,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -967,7 +967,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="10B981"/>
               </a:solidFill>
@@ -977,7 +977,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1002,7 +1002,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="1E40AF"/>
               </a:solidFill>
@@ -1012,7 +1012,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1037,7 +1037,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="F59E0B"/>
               </a:solidFill>
@@ -1047,7 +1047,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1072,7 +1072,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="EF4444"/>
               </a:solidFill>
@@ -1082,7 +1082,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1107,7 +1107,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
               <a:solidFill>
                 <a:srgbClr val="8B5CF6"/>
               </a:solidFill>
@@ -1117,7 +1117,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1146,8 +1146,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1184,7 +1184,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -1195,8 +1195,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1236,14 +1236,14 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1268,7 +1268,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1309,7 +1309,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -1320,8 +1320,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1361,14 +1361,14 @@
 </file>
 
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="11"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1393,10 +1393,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="10B981"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1420,10 +1420,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1E40AF"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1447,10 +1447,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="F59E0B"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1474,10 +1474,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EF4444"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1501,10 +1501,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="8B5CF6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1546,7 +1546,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -1557,8 +1557,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1598,14 +1598,14 @@
 </file>
 
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1630,7 +1630,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1671,7 +1671,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="4500">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4500">
               <a:solidFill>
                 <a:srgbClr val="D0D0D0"/>
               </a:solidFill>
@@ -1682,8 +1682,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1723,7 +1723,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -1738,9 +1738,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1750,7 +1750,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -1765,9 +1765,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1777,7 +1777,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -1792,9 +1792,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1804,7 +1804,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -1819,9 +1819,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1831,7 +1831,7 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -1846,9 +1846,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1858,7 +1858,7 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -1873,9 +1873,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1885,7 +1885,7 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -1900,9 +1900,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1912,7 +1912,7 @@
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -1927,9 +1927,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1939,7 +1939,7 @@
 </file>
 
 <file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1954,9 +1954,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="D48" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
@@ -3563,7 +3563,7 @@
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>Default classico 1,6% sul prospetto, a prezzo 102 con 5y residui → YTM ~1,2% reale.</t>
+          <t>Default classico 1,6% sul prospetto, a prezzo 102 con 4y residui → YTM ~1,1% reale.</t>
         </is>
       </c>
     </row>
@@ -5211,19 +5211,19 @@
         </is>
       </c>
       <c r="B6" s="16">
-        <f>'1 - Parametri'!B5*(1-'1 - Parametri'!B8)+('1 - Parametri'!B7)/5*(1-'1 - Parametri'!B8)</f>
+        <f>('1 - Parametri'!B5+('1 - Parametri'!B7)/5+'1 - Parametri'!B37)*(1-'1 - Parametri'!B8)-'1 - Parametri'!B37</f>
         <v/>
       </c>
       <c r="C6" s="16">
-        <f>'1 - Parametri'!B5*(1-'1 - Parametri'!B8)+('1 - Parametri'!B7)/5*(1-'1 - Parametri'!B8)</f>
+        <f>('1 - Parametri'!B5+('1 - Parametri'!B7)/5+'1 - Parametri'!B38)*(1-'1 - Parametri'!B8)-'1 - Parametri'!B38</f>
         <v/>
       </c>
       <c r="D6" s="16">
-        <f>'1 - Parametri'!B5*(1-'1 - Parametri'!B8)+('1 - Parametri'!B7)/5*(1-'1 - Parametri'!B8)</f>
+        <f>('1 - Parametri'!B5+('1 - Parametri'!B7)/5+'1 - Parametri'!B39)*(1-'1 - Parametri'!B8)-'1 - Parametri'!B39</f>
         <v/>
       </c>
       <c r="E6" s="16">
-        <f>'1 - Parametri'!B5*(1-'1 - Parametri'!B8)+('1 - Parametri'!B7)/5*(1-'1 - Parametri'!B8)</f>
+        <f>('1 - Parametri'!B5+('1 - Parametri'!B7)/5+'1 - Parametri'!B40)*(1-'1 - Parametri'!B8)-'1 - Parametri'!B40</f>
         <v/>
       </c>
     </row>
@@ -5234,19 +5234,19 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>'1 - Parametri'!B56*(1-'1 - Parametri'!B8)</f>
+        <f>'1 - Parametri'!B56*(1-'1 - Parametri'!B8)-'1 - Parametri'!B8*'1 - Parametri'!B37</f>
         <v/>
       </c>
       <c r="C7" s="16">
-        <f>'1 - Parametri'!B56*(1-'1 - Parametri'!B8)</f>
+        <f>'1 - Parametri'!B56*(1-'1 - Parametri'!B8)-'1 - Parametri'!B8*'1 - Parametri'!B38</f>
         <v/>
       </c>
       <c r="D7" s="16">
-        <f>'1 - Parametri'!B56*(1-'1 - Parametri'!B8)</f>
+        <f>'1 - Parametri'!B56*(1-'1 - Parametri'!B8)-'1 - Parametri'!B8*'1 - Parametri'!B39</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>'1 - Parametri'!B56*(1-'1 - Parametri'!B8)</f>
+        <f>'1 - Parametri'!B56*(1-'1 - Parametri'!B8)-'1 - Parametri'!B8*'1 - Parametri'!B40</f>
         <v/>
       </c>
     </row>
@@ -5449,7 +5449,7 @@
       </c>
       <c r="D5" s="20" t="inlineStr">
         <is>
-          <t>Soglia infl. break-even</t>
+          <t>Soglia infl. break-even (lorda)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -5473,7 +5473,7 @@
         <v/>
       </c>
       <c r="D6" s="16">
-        <f>C6-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)*(1-'1 - Parametri'!B8)</f>
+        <f>B6-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)</f>
         <v/>
       </c>
       <c r="E6" s="21">
@@ -5496,7 +5496,7 @@
         <v/>
       </c>
       <c r="D7" s="16">
-        <f>C7-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)*(1-'1 - Parametri'!B8)</f>
+        <f>B7-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)</f>
         <v/>
       </c>
       <c r="E7" s="21">
@@ -5519,7 +5519,7 @@
         <v/>
       </c>
       <c r="D8" s="16">
-        <f>C8-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)*(1-'1 - Parametri'!B8)</f>
+        <f>B8-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)</f>
         <v/>
       </c>
       <c r="E8" s="21">
@@ -5542,7 +5542,7 @@
         <v/>
       </c>
       <c r="D9" s="16">
-        <f>C9-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)*(1-'1 - Parametri'!B8)</f>
+        <f>B9-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)</f>
         <v/>
       </c>
       <c r="E9" s="21">
@@ -5565,7 +5565,7 @@
         <v/>
       </c>
       <c r="D10" s="16">
-        <f>C10-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)*(1-'1 - Parametri'!B8)</f>
+        <f>B10-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)</f>
         <v/>
       </c>
       <c r="E10" s="21">
@@ -5588,7 +5588,7 @@
         <v/>
       </c>
       <c r="D11" s="16">
-        <f>C11-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)*(1-'1 - Parametri'!B8)</f>
+        <f>B11-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)</f>
         <v/>
       </c>
       <c r="E11" s="21">
@@ -5611,7 +5611,7 @@
         <v/>
       </c>
       <c r="D12" s="16">
-        <f>C12-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)*(1-'1 - Parametri'!B8)</f>
+        <f>B12-('1 - Parametri'!B5+('1 - Parametri'!B7)/5)</f>
         <v/>
       </c>
       <c r="E12" s="21">

</xml_diff>

<commit_message>
@ Aggiunto foglio 12 "Switch" al simulatore BTP Italia Si
- Foglio Switch: conviene vendere un vecchio BTP Italia per il nuovo Si?
  Confronto rendimento reale forward + prezzo di indifferenza + verdetto.
- Grafico break-even (ScatterChart): due rette che si incrociano al prezzo
  di indifferenza, con label del valore sul punto.
- README aggiornato (11 -> 12 fogli).
@
</commit_message>
<xml_diff>
--- a/simulatori/btp_si_compare_2026.xlsx
+++ b/simulatori/btp_si_compare_2026.xlsx
@@ -19,6 +19,7 @@
     <sheet name="9 - 4 profili FIRE" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="10 - Calcolatore personale" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="11 - Flusso cedolare" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12 - Switch" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,12 +28,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000%"/>
     <numFmt numFmtId="167" formatCode="0.000%"/>
     <numFmt numFmtId="168" formatCode="mmm aaaa"/>
+    <numFmt numFmtId="169" formatCode="+0.00%;-0.00%;0.00%"/>
+    <numFmt numFmtId="170" formatCode="#,##0&quot; EUR&quot;"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -145,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -225,6 +228,12 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -542,6 +551,267 @@
         <crossAx val="10"/>
       </valAx>
     </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Break-even: quando conviene lo switch</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <scatterStyle val="lineMarker"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Vecchio (rend. reale)</v>
+          </tx>
+          <spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:srgbClr val="E0A458"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'12 - Switch'!$A$34:$A$41</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'12 - Switch'!$B$34:$B$41</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Nuovo Si (rend. reale)</v>
+          </tx>
+          <spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:srgbClr val="10B981"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'12 - Switch'!$A$34:$A$41</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'12 - Switch'!$C$34:$C$41</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Prezzo di indifferenza</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="diamond"/>
+            <size val="12"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="EF4444"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="0"/>
+              <tx>
+                <rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:r>
+                      <a:rPr lang="it-IT" b="1" sz="1150">
+                        <a:solidFill>
+                          <a:srgbClr val="C00000"/>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t>≈ 100,7</a:t>
+                    </a:r>
+                  </a:p>
+                </rich>
+              </tx>
+              <dLblPos val="t"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="0"/>
+              <showPercent val="0"/>
+              <showBubbleSize val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'12 - Switch'!$B$24</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'12 - Switch'!$B$14</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Prezzo del vecchio (su 100)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <layout>
+            <manualLayout>
+              <xMode val="edge"/>
+              <yMode val="edge"/>
+              <wMode val="factor"/>
+              <hMode val="factor"/>
+              <x val="0.4"/>
+              <y val="0.93"/>
+            </manualLayout>
+          </layout>
+          <overlay val="0"/>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="3000">
+              <a:solidFill>
+                <a:srgbClr val="ECECEC"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Rendimento reale annuo</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <layout>
+            <manualLayout>
+              <xMode val="edge"/>
+              <yMode val="edge"/>
+              <wMode val="factor"/>
+              <hMode val="factor"/>
+              <x val="0.005"/>
+              <y val="0.3"/>
+            </manualLayout>
+          </layout>
+          <overlay val="0"/>
+        </title>
+        <numFmt formatCode="0.0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+      <overlay val="0"/>
+    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -1948,6 +2218,33 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7560000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -3783,6 +4080,371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Switch: conviene vendere un vecchio BTP Italia per il nuovo Si?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Strumento informativo / divulgativo. NON è consulenza finanziaria. I valori sono indicativi al 2026 e vanno verificati col tuo consulente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Il tuo vecchio BTP Italia (quello che valuti di vendere)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Nominale posseduto (EUR)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Prezzo MOT attuale (su 100)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>101.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Tasso reale del vecchio (% annuo)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>0.0185</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Anni residui alla scadenza</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Il nuovo BTP Italia Si (in emissione, a 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Tasso reale</t>
+        </is>
+      </c>
+      <c r="B11" s="16">
+        <f>'1 - Parametri'!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Premio fedelta' (a scadenza)</t>
+        </is>
+      </c>
+      <c r="B12" s="16">
+        <f>'1 - Parametri'!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Durata (anni)</t>
+        </is>
+      </c>
+      <c r="B13" s="19">
+        <f>'1 - Parametri'!B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Rendimento reale annuo (comprato a 100)</t>
+        </is>
+      </c>
+      <c r="B14" s="16">
+        <f>B11+B12/B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Confronto: rendimento reale annuo DA OGGI</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Vecchio, tenuto a scadenza (sul prezzo attuale)</t>
+        </is>
+      </c>
+      <c r="B17" s="16">
+        <f>(B7*100+(100-B6)/B8)/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Nuovo Si (comprato a 100)</t>
+        </is>
+      </c>
+      <c r="B18" s="16">
+        <f>B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Differenza annua (Si - vecchio)</t>
+        </is>
+      </c>
+      <c r="B19" s="31">
+        <f>B18-B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Vantaggio stimato dello switch (su 5 anni)</t>
+        </is>
+      </c>
+      <c r="B20" s="32">
+        <f>B19*B13*(B5*B6/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Verdetto</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Conviene lo switch?</t>
+        </is>
+      </c>
+      <c r="B23" s="25">
+        <f>IF(B18&gt;B17,"SI - valuta lo switch","NO - tieni il vecchio")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Prezzo di indifferenza del vecchio</t>
+        </is>
+      </c>
+      <c r="B24" s="24">
+        <f>(B7*100+100/B8)/(B18+1/B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Logica: confronta il rendimento reale annuo che otterresti DA OGGI tenendo il vecchio (penalizzato se quota sopra 100, perche' a scadenza torna a 100) contro il Si comprato a 100. Se il vecchio quota SOPRA il prezzo di indifferenza, lo switch inizia ad avere senso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Attenzione: vendendo il vecchio perdi il rateo/rivalutazione gia' maturati e il suo premio fedelta'; paghi spread ed esecuzione. Per piccoli importi il vantaggio e' spesso di pochi euro. Stima semplificata (rendimento 'semplice', cedole non reinvestite). NON e' consulenza finanziaria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Dati grafico break-even (prezzo del vecchio -&gt; rendimento reale)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>Prezzo vecchio</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>Vecchio (rend. reale)</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>Nuovo Si (rend. reale)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="n">
+        <v>98</v>
+      </c>
+      <c r="B34" s="16">
+        <f>(B$7*100+(100-A34)/B$8)/A34</f>
+        <v/>
+      </c>
+      <c r="C34" s="16">
+        <f>B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="n">
+        <v>99</v>
+      </c>
+      <c r="B35" s="16">
+        <f>(B$7*100+(100-A35)/B$8)/A35</f>
+        <v/>
+      </c>
+      <c r="C35" s="16">
+        <f>B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="B36" s="16">
+        <f>(B$7*100+(100-A36)/B$8)/A36</f>
+        <v/>
+      </c>
+      <c r="C36" s="16">
+        <f>B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="n">
+        <v>101</v>
+      </c>
+      <c r="B37" s="16">
+        <f>(B$7*100+(100-A37)/B$8)/A37</f>
+        <v/>
+      </c>
+      <c r="C37" s="16">
+        <f>B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="n">
+        <v>102</v>
+      </c>
+      <c r="B38" s="16">
+        <f>(B$7*100+(100-A38)/B$8)/A38</f>
+        <v/>
+      </c>
+      <c r="C38" s="16">
+        <f>B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="n">
+        <v>103</v>
+      </c>
+      <c r="B39" s="16">
+        <f>(B$7*100+(100-A39)/B$8)/A39</f>
+        <v/>
+      </c>
+      <c r="C39" s="16">
+        <f>B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="n">
+        <v>104</v>
+      </c>
+      <c r="B40" s="16">
+        <f>(B$7*100+(100-A40)/B$8)/A40</f>
+        <v/>
+      </c>
+      <c r="C40" s="16">
+        <f>B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="n">
+        <v>105</v>
+      </c>
+      <c r="B41" s="16">
+        <f>(B$7*100+(100-A41)/B$8)/A41</f>
+        <v/>
+      </c>
+      <c r="C41" s="16">
+        <f>B$14</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Allinea prezzi MOT classico al 19/06 (mar2028 101,32 / giu2030 100,94) coerenti con web/JSON; label Switch come testo statico
</commit_message>
<xml_diff>
--- a/simulatori/btp_si_compare_2026.xlsx
+++ b/simulatori/btp_si_compare_2026.xlsx
@@ -559,7 +559,6 @@
 
 <file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="13"/>
   <chart>
     <title>
       <tx>
@@ -4919,7 +4918,7 @@
         </is>
       </c>
       <c r="B46" s="14" t="n">
-        <v>101.83</v>
+        <v>101.32</v>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
@@ -4943,7 +4942,7 @@
         </is>
       </c>
       <c r="B48" s="14" t="n">
-        <v>101.86</v>
+        <v>100.94</v>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>

</xml_diff>